<commit_message>
Cambio en menu principal
</commit_message>
<xml_diff>
--- a/TablasBaseDeDatos.xlsx
+++ b/TablasBaseDeDatos.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documentos\ProgramaciónWeb\ProyectoRegistroAnimal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED73F7F-BC24-45C2-914A-7A88C5C19F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D183A6-7CD7-4082-8426-0ACD4D920C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
   </bookViews>
   <sheets>
     <sheet name="Animal" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Dueño" sheetId="2" r:id="rId2"/>
+    <sheet name="Trabajador" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="33">
   <si>
     <t>Tipo</t>
   </si>
@@ -101,28 +102,40 @@
     <t>Curp</t>
   </si>
   <si>
-    <t>Fecha de nacimiento</t>
-  </si>
-  <si>
-    <t>Estado civil</t>
-  </si>
-  <si>
     <t>Telefono</t>
   </si>
   <si>
-    <t>Correo electronico</t>
-  </si>
-  <si>
     <t>Direccion</t>
   </si>
   <si>
     <t>Id dueño</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
     <t>Varchar(10) Not null</t>
+  </si>
+  <si>
+    <t>Apellido paterno</t>
+  </si>
+  <si>
+    <t>Apellido materno</t>
+  </si>
+  <si>
+    <t>Correo electrónico</t>
+  </si>
+  <si>
+    <t>Nombre(s)</t>
+  </si>
+  <si>
+    <t>Varchar(255) Not null</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>Lo usuarios no ven esto, es para identificarlos dentro del sistema</t>
+  </si>
+  <si>
+    <t>Clave catastral</t>
   </si>
 </sst>
 </file>
@@ -578,7 +591,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{084CE3D9-1975-40D0-BC88-39A1AE4F9789}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -592,18 +605,24 @@
       <c r="B1" t="s">
         <v>0</v>
       </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -611,62 +630,116 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C15" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB4FE8CD-86E0-44ED-81E8-12936ADBB839}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>25</v>
       </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C13" s="1"/>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambios en registroTrabajadores.html, se agrego funcion de generar password aleatorias con registrotrabajadores.js
</commit_message>
<xml_diff>
--- a/TablasBaseDeDatos.xlsx
+++ b/TablasBaseDeDatos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documentos\ProgramaciónWeb\ProyectoRegistroAnimal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D183A6-7CD7-4082-8426-0ACD4D920C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90CD699-EE2E-48B8-906A-AB5AFF9BA538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
   </bookViews>
   <sheets>
     <sheet name="Animal" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="41">
   <si>
     <t>Tipo</t>
   </si>
@@ -48,9 +48,6 @@
     <t>CurpDelDueño</t>
   </si>
   <si>
-    <t>NumAnimal</t>
-  </si>
-  <si>
     <t>Raza</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>Char(18) Not null</t>
   </si>
   <si>
-    <t>Int Not null Auto_increment</t>
-  </si>
-  <si>
     <t>Varchar(45) Not null</t>
   </si>
   <si>
@@ -90,15 +84,6 @@
     <t>Longtext Not null</t>
   </si>
   <si>
-    <t>Char(2) Not null Default('D')</t>
-  </si>
-  <si>
-    <t>Char(2) Not null Default('No')</t>
-  </si>
-  <si>
-    <t>Char(2) Not null Default('Si')</t>
-  </si>
-  <si>
     <t>Curp</t>
   </si>
   <si>
@@ -136,6 +121,45 @@
   </si>
   <si>
     <t>Clave catastral</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Int Not null Auto_increment primary key</t>
+  </si>
+  <si>
+    <t>Enum ("F","M","D") Not null Default('D')</t>
+  </si>
+  <si>
+    <t>Enum ("Si","No") Not null Default('No')</t>
+  </si>
+  <si>
+    <t>Contraseña</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>Enum (Ofc, Cns, Adm), Not null</t>
+  </si>
+  <si>
+    <t>Created_at</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Current_timestamp</t>
+  </si>
+  <si>
+    <t>is_active</t>
+  </si>
+  <si>
+    <t>TinyInt Not null</t>
+  </si>
+  <si>
+    <t>1'</t>
   </si>
 </sst>
 </file>
@@ -171,9 +195,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,15 +513,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E44CD059-3547-42F8-B933-AB464B95C06B}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -504,84 +529,109 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
       <c r="B3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -595,7 +645,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,74 +656,96 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -686,59 +758,111 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB4FE8CD-86E0-44ED-81E8-12936ADBB839}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambios generales en proyecto
</commit_message>
<xml_diff>
--- a/TablasBaseDeDatos.xlsx
+++ b/TablasBaseDeDatos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files (x86)\EasyPHP-Devserver-17\eds-www\ProyectoRegistroAnimal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93843846-BAE4-4698-A081-5BE6AC2E9262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4602332-D016-4161-8763-DCCE6B5E9AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C8ADCFF7-7EDB-42C1-B28A-DEEC49684928}"/>
   </bookViews>
   <sheets>
     <sheet name="Animal" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
   <si>
     <t>Tipo</t>
   </si>
@@ -119,9 +119,6 @@
   </si>
   <si>
     <t>Lo usuarios no ven esto, es para identificarlos dentro del sistema</t>
-  </si>
-  <si>
-    <t>Clave catastral</t>
   </si>
   <si>
     <t>ID</t>
@@ -538,10 +535,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -600,7 +597,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -608,7 +605,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -616,29 +613,29 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -648,7 +645,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{084CE3D9-1975-40D0-BC88-39A1AE4F9789}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -671,7 +668,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -727,36 +724,28 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="A10" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C15" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C14" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -785,10 +774,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -836,7 +825,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -844,32 +833,32 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
         <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -899,10 +888,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
@@ -918,7 +907,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
@@ -926,7 +915,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>

</xml_diff>